<commit_message>
Update tên mặt hàng
</commit_message>
<xml_diff>
--- a/Data/BVMT.xlsx
+++ b/Data/BVMT.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Works 2\IT\GITHUB\UpSSE_BB\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BE2E5E94-9474-43EB-8A7A-CCD62205B7F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BA51ECB-FFAF-4011-BD62-F4B0464DB6BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2505" yWindow="2505" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet4" sheetId="4" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Tên mặt hàng</t>
   </si>
@@ -55,6 +54,9 @@
   </si>
   <si>
     <t>Dầu Điêzen 0,001S Mức 5</t>
+  </si>
+  <si>
+    <t>Xăng E10 RON 92 Mức 3</t>
   </si>
 </sst>
 </file>
@@ -377,7 +379,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B5"/>
+  <dimension ref="A1:B6"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.125" style="1" bestFit="1" customWidth="1"/>
@@ -425,6 +427,14 @@
         <v>1000</v>
       </c>
     </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1">
+        <v>1900</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>

</xml_diff>